<commit_message>
Refactor mailer and scheduler services for improved error logging and path handling
</commit_message>
<xml_diff>
--- a/sample - Copy.xlsx
+++ b/sample - Copy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f80e6e0943a1a34c/Desktop/Email Tool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="11_79C3E2171C397D6A206102A720D19643A12CC1D0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{858D3A97-AA60-4AF4-B35F-EDE6805D39E5}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="11_79C3E2171C397D6A206102A720D19643A12CC1D0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3CDD836-F6FE-4BEC-89C9-B59519960048}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
     <t>phone</t>
   </si>
   <si>
-    <t>Tue 16:53</t>
+    <t>Tue 17:09</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Enhance mailer transport configuration with Gmail settings and timeout options
</commit_message>
<xml_diff>
--- a/sample - Copy.xlsx
+++ b/sample - Copy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f80e6e0943a1a34c/Desktop/Email Tool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="11_79C3E2171C397D6A206102A720D19643A12CC1D0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3CDD836-F6FE-4BEC-89C9-B59519960048}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="11_79C3E2171C397D6A206102A720D19643A12CC1D0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BA42B0B-9BB1-438A-A334-BA3BD3FB4E23}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
     <t>phone</t>
   </si>
   <si>
-    <t>Tue 17:09</t>
+    <t>Tue 17:21</t>
   </si>
 </sst>
 </file>

</xml_diff>